<commit_message>
Update BHP holding to 11065 shares
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260715.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260715.xlsx
@@ -580,13 +580,13 @@
         </is>
       </c>
       <c r="E7" s="3" t="n">
-        <v>9000</v>
+        <v>11065</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>545040</v>
+        <v>670096.4</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>16650</v>
+        <v>20470.25</v>
       </c>
     </row>
     <row r="8">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1415990.14</v>
+        <v>1541046.54</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>14095.53</v>
+        <v>17915.78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>